<commit_message>
Add SDM Phase 2 employees to the portal with product tests and login workbooks.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Employee_User_Credentials.xlsx
+++ b/Employee_User_Credentials.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I266"/>
+  <dimension ref="A1:I289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4323,7 +4323,6 @@
           <t>sanjay_gupta.gupta.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -4366,7 +4365,6 @@
           <t>bharanidharan.sampath.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -4409,7 +4407,6 @@
           <t>afridi.afridi.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -4452,7 +4449,6 @@
           <t>divyanshu.chauhan.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -4495,7 +4491,6 @@
           <t>chitrangada.mishra.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -4538,7 +4533,6 @@
           <t>vibhor.gupta.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -4581,7 +4575,6 @@
           <t>nishu.kumar.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -4624,7 +4617,6 @@
           <t>satheesh.2.kumar.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -4667,7 +4659,6 @@
           <t>chandan.k.singh.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -4710,7 +4701,6 @@
           <t>sourabh.khandelwal.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -4753,7 +4743,6 @@
           <t>prateek.1.prateek.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -4796,7 +4785,6 @@
           <t>veerasami.m.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -4839,7 +4827,6 @@
           <t>parth.1.saxena.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -4882,7 +4869,6 @@
           <t>satya.rai.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -4925,7 +4911,6 @@
           <t>meenatchi.m.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -4968,7 +4953,6 @@
           <t>sunilkumaar.ts.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5011,7 +4995,6 @@
           <t>ashwini.r.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5054,7 +5037,6 @@
           <t>sunil.patel.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5097,7 +5079,6 @@
           <t>naveenkumar.murugan.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5140,7 +5121,6 @@
           <t>koushik.gunasekaran.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5183,7 +5163,6 @@
           <t>kapil.chaudhary.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5226,7 +5205,6 @@
           <t>aryan.kumar.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5269,7 +5247,6 @@
           <t>pratik.raj.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5312,7 +5289,6 @@
           <t>ezhilarasan.balasubramaniyan.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5355,7 +5331,6 @@
           <t>santhosh.5.kumar.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5398,7 +5373,6 @@
           <t>srinath.balasubramanian.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5441,7 +5415,6 @@
           <t>kiruthika.vinayagam.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5484,7 +5457,6 @@
           <t>pratyasa.mohanty.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5527,7 +5499,6 @@
           <t>soumya_smruti.das.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5570,7 +5541,6 @@
           <t>pratyusha.pattanaik.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5613,7 +5583,6 @@
           <t>ashutosh.2.mishra.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5656,7 +5625,6 @@
           <t>lakshmi.gudluru.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5699,7 +5667,6 @@
           <t>madanuru.charan.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5742,7 +5709,6 @@
           <t>mohanty.abhisek.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5785,7 +5751,6 @@
           <t>avipsa.mohanty.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5828,7 +5793,6 @@
           <t>debasish.jena.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5871,7 +5835,6 @@
           <t>pritisarathi.bhuyan.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5914,7 +5877,6 @@
           <t>anchal.swain.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -5957,7 +5919,6 @@
           <t>sasmita.giri.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6000,7 +5961,6 @@
           <t>akankshya.rout.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6043,7 +6003,6 @@
           <t>ajaya.nayak.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6086,7 +6045,6 @@
           <t>soumya.das.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6129,7 +6087,6 @@
           <t>vaghela.rahul.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
       <c r="F125" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6172,7 +6129,6 @@
           <t>ashis.nayak.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr"/>
       <c r="F126" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6215,7 +6171,6 @@
           <t>bibhash.dash.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6258,7 +6213,6 @@
           <t>omm.ranjan.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr"/>
       <c r="F128" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6301,7 +6255,6 @@
           <t>pradyumna.naik.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6344,7 +6297,6 @@
           <t>abdul.shaik.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6387,7 +6339,6 @@
           <t>jigar.solanki.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6430,7 +6381,6 @@
           <t>akash.bairagi.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6473,7 +6423,6 @@
           <t>anand.babu_s.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6516,7 +6465,6 @@
           <t>chelsea.shalin_s.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6559,7 +6507,6 @@
           <t>gopi.1.k.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6602,7 +6549,6 @@
           <t>malan.subbiah_pandian.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6645,7 +6591,6 @@
           <t>krishna.durga_r.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr"/>
       <c r="F137" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6688,7 +6633,6 @@
           <t>sabari.murugesan.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6731,7 +6675,6 @@
           <t>surya.1.saravanan.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6774,7 +6717,6 @@
           <t>yoga.verma_v.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr"/>
       <c r="F140" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6817,7 +6759,6 @@
           <t>varun.pachauri.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6860,7 +6801,6 @@
           <t>buran.sagari_sohail_basha.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6903,7 +6843,6 @@
           <t>yaswanth.gadde.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr"/>
       <c r="F143" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6946,7 +6885,6 @@
           <t>hariharan.1.s.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E144" t="inlineStr"/>
       <c r="F144" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -6989,7 +6927,6 @@
           <t>subramanyam.muddisetti.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E145" t="inlineStr"/>
       <c r="F145" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7032,7 +6969,6 @@
           <t>mahendra.nekkanti.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr"/>
       <c r="F146" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7075,7 +7011,6 @@
           <t>sandhiya.v_p.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr"/>
       <c r="F147" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7118,7 +7053,6 @@
           <t>susheel.k.dwivedi.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr"/>
       <c r="F148" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7161,7 +7095,6 @@
           <t>vivek.7.mishra.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7204,7 +7137,6 @@
           <t>harshada.vitthal_shinde.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7247,7 +7179,6 @@
           <t>nishant.lal.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr"/>
       <c r="F151" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7290,7 +7221,6 @@
           <t>vennela.korada.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E152" t="inlineStr"/>
       <c r="F152" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7333,7 +7263,6 @@
           <t>bommireddy.prakash_reddy.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7376,7 +7305,6 @@
           <t>komala.mamidi.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E154" t="inlineStr"/>
       <c r="F154" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7419,7 +7347,6 @@
           <t>sundram.kumar.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr"/>
       <c r="F155" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7462,7 +7389,6 @@
           <t>abhishikha.chauhan.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E156" t="inlineStr"/>
       <c r="F156" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7505,7 +7431,6 @@
           <t>anipeddi.lasya.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr"/>
       <c r="F157" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7548,7 +7473,6 @@
           <t>biruntha.biruntha.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E158" t="inlineStr"/>
       <c r="F158" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7591,7 +7515,6 @@
           <t>himanshu.1.bungla.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E159" t="inlineStr"/>
       <c r="F159" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7634,7 +7557,6 @@
           <t>nijampatnam.eswar.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E160" t="inlineStr"/>
       <c r="F160" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7677,7 +7599,6 @@
           <t>saiyed.imam.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E161" t="inlineStr"/>
       <c r="F161" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7720,7 +7641,6 @@
           <t>vaijinath.batule.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7763,7 +7683,6 @@
           <t>kamal.k.ray.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7806,7 +7725,6 @@
           <t>tanmoy.mojumder.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E164" t="inlineStr"/>
       <c r="F164" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7849,7 +7767,6 @@
           <t>reshma.shaikh.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E165" t="inlineStr"/>
       <c r="F165" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7892,7 +7809,6 @@
           <t>om.gautam.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E166" t="inlineStr"/>
       <c r="F166" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7935,7 +7851,6 @@
           <t>jaya.vohra.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E167" t="inlineStr"/>
       <c r="F167" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -7978,7 +7893,6 @@
           <t>bijetananda.swain.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E168" t="inlineStr"/>
       <c r="F168" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8021,7 +7935,6 @@
           <t>rohit.18.kumar.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E169" t="inlineStr"/>
       <c r="F169" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8064,7 +7977,6 @@
           <t>sujata.singh.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E170" t="inlineStr"/>
       <c r="F170" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8107,7 +8019,6 @@
           <t>sushma.cholleti.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E171" t="inlineStr"/>
       <c r="F171" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8150,7 +8061,6 @@
           <t>gaurav.verma.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E172" t="inlineStr"/>
       <c r="F172" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8193,7 +8103,6 @@
           <t>kamna.peyal.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E173" t="inlineStr"/>
       <c r="F173" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8236,7 +8145,6 @@
           <t>vinay.damarasinghu.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E174" t="inlineStr"/>
       <c r="F174" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8279,7 +8187,6 @@
           <t>srivalli.devarapalli_siva.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E175" t="inlineStr"/>
       <c r="F175" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8322,7 +8229,6 @@
           <t>srinivas.chandan_etakaati.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E176" t="inlineStr"/>
       <c r="F176" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8365,7 +8271,6 @@
           <t>vaishnavi.guttula.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E177" t="inlineStr"/>
       <c r="F177" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8408,7 +8313,6 @@
           <t>hamsa.yaswanth_paul.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E178" t="inlineStr"/>
       <c r="F178" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8451,7 +8355,6 @@
           <t>nandini.kasi.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E179" t="inlineStr"/>
       <c r="F179" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8494,7 +8397,6 @@
           <t>lavanya.seerapu.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E180" t="inlineStr"/>
       <c r="F180" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8537,7 +8439,6 @@
           <t>sai.pappala.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E181" t="inlineStr"/>
       <c r="F181" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8580,7 +8481,6 @@
           <t>deepthisri.rachabathula.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8623,7 +8523,6 @@
           <t>srujan.palla.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E183" t="inlineStr"/>
       <c r="F183" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8666,7 +8565,6 @@
           <t>swetha.konchada.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E184" t="inlineStr"/>
       <c r="F184" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8709,7 +8607,6 @@
           <t>vivek.3.singh.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E185" t="inlineStr"/>
       <c r="F185" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8752,7 +8649,6 @@
           <t>akshit.sahni.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E186" t="inlineStr"/>
       <c r="F186" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8795,7 +8691,6 @@
           <t>abhiram.jagarlamudi.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E187" t="inlineStr"/>
       <c r="F187" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8838,7 +8733,6 @@
           <t>debopriyo.halder.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E188" t="inlineStr"/>
       <c r="F188" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8881,7 +8775,6 @@
           <t>alok.nayak.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E189" t="inlineStr"/>
       <c r="F189" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8924,7 +8817,6 @@
           <t>archit.bagulia.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E190" t="inlineStr"/>
       <c r="F190" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -8967,7 +8859,6 @@
           <t>arunkumar.pattadakall.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E191" t="inlineStr"/>
       <c r="F191" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9010,7 +8901,6 @@
           <t>dewashish.kumar.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E192" t="inlineStr"/>
       <c r="F192" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9053,7 +8943,6 @@
           <t>subhankar.hazra.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E193" t="inlineStr"/>
       <c r="F193" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9096,7 +8985,6 @@
           <t>ajay.17.kumar.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E194" t="inlineStr"/>
       <c r="F194" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9139,7 +9027,6 @@
           <t>altamash.ashfaq.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E195" t="inlineStr"/>
       <c r="F195" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9182,7 +9069,6 @@
           <t>preetam.mehta.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E196" t="inlineStr"/>
       <c r="F196" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9225,7 +9111,6 @@
           <t>guru.prasad.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E197" t="inlineStr"/>
       <c r="F197" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9268,7 +9153,6 @@
           <t>raviraj.chalikwar.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E198" t="inlineStr"/>
       <c r="F198" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9311,7 +9195,6 @@
           <t>snehal.mavale.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E199" t="inlineStr"/>
       <c r="F199" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9354,7 +9237,6 @@
           <t>rakshitha.k_m.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E200" t="inlineStr"/>
       <c r="F200" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9397,7 +9279,6 @@
           <t>sakshi.3.srivastava.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E201" t="inlineStr"/>
       <c r="F201" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9440,7 +9321,6 @@
           <t>sukanya.avvari.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E202" t="inlineStr"/>
       <c r="F202" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9483,7 +9363,6 @@
           <t>vijay.dhomase.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E203" t="inlineStr"/>
       <c r="F203" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9526,7 +9405,6 @@
           <t>angshuman.sarma.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E204" t="inlineStr"/>
       <c r="F204" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9569,7 +9447,6 @@
           <t>nisha.mali.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E205" t="inlineStr"/>
       <c r="F205" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9612,7 +9489,6 @@
           <t>ravi.8.ranjan.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E206" t="inlineStr"/>
       <c r="F206" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9655,7 +9531,6 @@
           <t>sarjitkumar.rajyaguru.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E207" t="inlineStr"/>
       <c r="F207" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9698,7 +9573,6 @@
           <t>ajith.v_a.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E208" t="inlineStr"/>
       <c r="F208" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9741,7 +9615,6 @@
           <t>sugat.bhalshankar.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E209" t="inlineStr"/>
       <c r="F209" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9784,7 +9657,6 @@
           <t>altaf.ahmad.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E210" t="inlineStr"/>
       <c r="F210" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9827,7 +9699,6 @@
           <t>dhruv.kant_goyal.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E211" t="inlineStr"/>
       <c r="F211" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9870,7 +9741,6 @@
           <t>ayyub.mohammad.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E212" t="inlineStr"/>
       <c r="F212" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9913,7 +9783,6 @@
           <t>vivek.8.mishra.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E213" t="inlineStr"/>
       <c r="F213" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9956,7 +9825,6 @@
           <t>abhishek.k.patel.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E214" t="inlineStr"/>
       <c r="F214" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -9999,7 +9867,6 @@
           <t>chandra.sen.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E215" t="inlineStr"/>
       <c r="F215" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10042,7 +9909,6 @@
           <t>depankar.kumar.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E216" t="inlineStr"/>
       <c r="F216" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10085,7 +9951,6 @@
           <t>mohanram.g.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E217" t="inlineStr"/>
       <c r="F217" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10128,7 +9993,6 @@
           <t>manpreet.2.kaur.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E218" t="inlineStr"/>
       <c r="F218" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10171,7 +10035,6 @@
           <t>timmappa.r.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E219" t="inlineStr"/>
       <c r="F219" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10214,7 +10077,6 @@
           <t>smruti.s.sahoo.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E220" t="inlineStr"/>
       <c r="F220" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10257,7 +10119,6 @@
           <t>tejaswini.patel.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E221" t="inlineStr"/>
       <c r="F221" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10300,7 +10161,6 @@
           <t>amit.ghadge.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E222" t="inlineStr"/>
       <c r="F222" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10343,7 +10203,6 @@
           <t>sayanth.a_v.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E223" t="inlineStr"/>
       <c r="F223" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10386,7 +10245,6 @@
           <t>abhishek.22.kumar.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E224" t="inlineStr"/>
       <c r="F224" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10429,7 +10287,6 @@
           <t>avinash.1.yadav.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E225" t="inlineStr"/>
       <c r="F225" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10472,7 +10329,6 @@
           <t>mdaliahmed.jameel.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E226" t="inlineStr"/>
       <c r="F226" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10515,7 +10371,6 @@
           <t>mohammad.m.khan.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E227" t="inlineStr"/>
       <c r="F227" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10558,7 +10413,6 @@
           <t>nirosha.naredla.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E228" t="inlineStr"/>
       <c r="F228" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10601,7 +10455,6 @@
           <t>sachin.gilbile.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E229" t="inlineStr"/>
       <c r="F229" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10644,7 +10497,6 @@
           <t>liji.babu.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E230" t="inlineStr"/>
       <c r="F230" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10687,7 +10539,6 @@
           <t>arvind.k2.singh.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E231" t="inlineStr"/>
       <c r="F231" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10730,7 +10581,6 @@
           <t>aparajita.shankar.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E232" t="inlineStr"/>
       <c r="F232" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10773,7 +10623,6 @@
           <t>phani.datta.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E233" t="inlineStr"/>
       <c r="F233" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10816,7 +10665,6 @@
           <t>mohan.1.kumar.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E234" t="inlineStr"/>
       <c r="F234" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10859,7 +10707,6 @@
           <t>manoj.kannan.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E235" t="inlineStr"/>
       <c r="F235" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10902,7 +10749,6 @@
           <t>supraja.srivani.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E236" t="inlineStr"/>
       <c r="F236" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10945,7 +10791,6 @@
           <t>nutan.1.rani.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E237" t="inlineStr"/>
       <c r="F237" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -10988,7 +10833,6 @@
           <t>prasanth.subramaniyan.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E238" t="inlineStr"/>
       <c r="F238" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11031,7 +10875,6 @@
           <t>pankaj.1.verma.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E239" t="inlineStr"/>
       <c r="F239" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11074,7 +10917,6 @@
           <t>madhura.atul_kulkarni.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E240" t="inlineStr"/>
       <c r="F240" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11117,7 +10959,6 @@
           <t>sahil.mantrao.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E241" t="inlineStr"/>
       <c r="F241" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11160,7 +11001,6 @@
           <t>satish.maurya.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E242" t="inlineStr"/>
       <c r="F242" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11203,7 +11043,6 @@
           <t>janardan.singh.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E243" t="inlineStr"/>
       <c r="F243" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11246,7 +11085,6 @@
           <t>kushagra.chaudhary.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E244" t="inlineStr"/>
       <c r="F244" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11289,7 +11127,6 @@
           <t>ayan.roy.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E245" t="inlineStr"/>
       <c r="F245" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11332,7 +11169,6 @@
           <t>yashi.gupta.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E246" t="inlineStr"/>
       <c r="F246" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11375,7 +11211,6 @@
           <t>anita.km.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E247" t="inlineStr"/>
       <c r="F247" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11418,7 +11253,6 @@
           <t>Nitesh.3.kumar.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E248" t="inlineStr"/>
       <c r="F248" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11461,7 +11295,6 @@
           <t>Pratibha.1.singh.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E249" t="inlineStr"/>
       <c r="F249" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11504,7 +11337,6 @@
           <t>neha.ojha.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E250" t="inlineStr"/>
       <c r="F250" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11547,7 +11379,6 @@
           <t>p.vishnu.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E251" t="inlineStr"/>
       <c r="F251" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11590,7 +11421,6 @@
           <t>khusboo.mantoo.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E252" t="inlineStr"/>
       <c r="F252" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11633,7 +11463,6 @@
           <t>shridhar.patange.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E253" t="inlineStr"/>
       <c r="F253" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11676,7 +11505,6 @@
           <t>vishal.2.chaudhary.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E254" t="inlineStr"/>
       <c r="F254" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11719,7 +11547,6 @@
           <t>niteesh.pandey.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E255" t="inlineStr"/>
       <c r="F255" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11762,7 +11589,6 @@
           <t>akanksha.haste.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E256" t="inlineStr"/>
       <c r="F256" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11805,7 +11631,6 @@
           <t>abdullah.farooqi.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E257" t="inlineStr"/>
       <c r="F257" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11848,7 +11673,6 @@
           <t>devendra.gupta.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E258" t="inlineStr"/>
       <c r="F258" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11891,7 +11715,6 @@
           <t>mukkollu.nagababu.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E259" t="inlineStr"/>
       <c r="F259" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11934,7 +11757,6 @@
           <t>divyanshu.bhadouria.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E260" t="inlineStr"/>
       <c r="F260" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -11977,7 +11799,6 @@
           <t>harshraj.sharma.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E261" t="inlineStr"/>
       <c r="F261" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -12020,7 +11841,6 @@
           <t>deepak.k1.sharma.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E262" t="inlineStr"/>
       <c r="F262" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -12063,7 +11883,6 @@
           <t>anand.2.kumar.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E263" t="inlineStr"/>
       <c r="F263" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -12106,7 +11925,6 @@
           <t>priya.mani.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E264" t="inlineStr"/>
       <c r="F264" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -12149,7 +11967,6 @@
           <t>navyasri.neelapu.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E265" t="inlineStr"/>
       <c r="F265" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -12192,7 +12009,6 @@
           <t>deepika.subburaj.ext@nokia.com</t>
         </is>
       </c>
-      <c r="E266" t="inlineStr"/>
       <c r="F266" t="inlineStr">
         <is>
           <t>PACO</t>
@@ -12211,6 +12027,1087 @@
       <c r="I266" t="inlineStr">
         <is>
           <t>Kalia</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>1035501</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Omkar</t>
+        </is>
+      </c>
+      <c r="C267" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Omkar5501</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>omkar.singh.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>HLR-HSS</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>FASTWEB</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>Sugandh Sinha</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>1034806</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>M Ashok Kumar</t>
+        </is>
+      </c>
+      <c r="C268" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Ashok4806</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>ashok.kumar_m.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>HLR-HSS</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>3UK</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>Sugandh Sinha</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>1034813</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Naveen Kumar B</t>
+        </is>
+      </c>
+      <c r="C269" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Naveen4813</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>naveen.kumar_b.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>HLR-HSS</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>Sugandh Sinha</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>1039139</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Bobbarala Varshitha</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Bobbarala9139</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>bobbarala.varshitha.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>HLR-HSS</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>ORANGE</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>Sugandh Sinha</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>1040910</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Ravi Shankar</t>
+        </is>
+      </c>
+      <c r="C271" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Ravi0910</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>ravi.s.sharma.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>HLR-HSS</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>Kite</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>Sugandh Sinha</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>1037017</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Adarsh Putta</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Adarsh7017</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>putta.adarsh.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>HLR-HSS</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>Sugandh Sinha</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>1042582</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Mamidi Jyothsna</t>
+        </is>
+      </c>
+      <c r="C273" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Mamidi2582</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>jyothsna.mamidi.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>HLR-HSS</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>Sugandh Sinha</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>1035564</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Abhinav Maheshwari</t>
+        </is>
+      </c>
+      <c r="C274" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Abhinav5564</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>abhinav.maheshwari.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>EIR</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>3UK</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>Mahendra Rajput</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>1035300</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Ashwini S</t>
+        </is>
+      </c>
+      <c r="C275" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Ashwini5300</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>ashwini.selvaraj.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>EIR</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>3UK</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>Mahendra Rajput</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>1041595</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Manisha Ganpat Lohar</t>
+        </is>
+      </c>
+      <c r="C276" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Manisha1595</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>manisha.lohar.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>EIR</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>FASTWEB</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>Mahendra Rajput</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>1041603</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Aniket Nagdeve</t>
+        </is>
+      </c>
+      <c r="C277" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Aniket1603</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>aniket.nagdeve.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>EIR</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>3UK</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>Mahendra Rajput</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>1041246</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Sushree Ranjita Panda</t>
+        </is>
+      </c>
+      <c r="C278" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Sushree1246</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>sushree.ranjita_panda.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>EIR</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>ORANGE</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>Mahendra Rajput</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>1039152</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Sadhana S</t>
+        </is>
+      </c>
+      <c r="C279" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Sadhana9152</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>sadhana.s.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>UDM</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>Aramco</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>Emmanual</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>1035997</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Sri Gokula Karthikeyan</t>
+        </is>
+      </c>
+      <c r="C280" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Sri5997</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>gokula.karthikeyan.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>UDM</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>Emmanual</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>1042552</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Apurva Anil Patil</t>
+        </is>
+      </c>
+      <c r="C281" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Apurva2552</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>apurva_anil_patil.patil.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>SDL</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>EE BT</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>Dinil</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>1039120</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Manish Thukral</t>
+        </is>
+      </c>
+      <c r="C282" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Manish9120</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>manish.thukral.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>SDL</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>Turk telecom</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>Dinil</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>1039793</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Ginni Sinha</t>
+        </is>
+      </c>
+      <c r="C283" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Ginni9793</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>ginni.sinha.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>SDL</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>PROXIMUS</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>Dinil</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>1042167</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Subhasantosh Dash</t>
+        </is>
+      </c>
+      <c r="C284" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Subhasantosh2167</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>subhasantosh.dash.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>SDL</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>Dinil</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>1034349</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Yash Khurana</t>
+        </is>
+      </c>
+      <c r="C285" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Yash4349</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>yash.khurana.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>SDL</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>BSI</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>Dinil</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>1706842</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Amlan Ashish Sahoo</t>
+        </is>
+      </c>
+      <c r="C286" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Amlan6842</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>amlan.sahoo.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>SDL</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>EE BT</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>Dinil</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>1042388</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Manjunath U H</t>
+        </is>
+      </c>
+      <c r="C287" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Manjunath2388</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>manjunath.u_h.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>SDL</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>AIRE</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>Dinil</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>1035777</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Sobhika R</t>
+        </is>
+      </c>
+      <c r="C288" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Sobhika5777</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>sobhika.rajkumar.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>SDL</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>Telemech</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>Dinil</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>1034275</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Onkar Sharma</t>
+        </is>
+      </c>
+      <c r="C289" s="2" t="inlineStr">
+        <is>
+          <t>EMP@Onkar4275</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>onkar.sharma.ext@nokia.com</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Solution Engineer</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>SDL</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>PROXIMUS</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>Dinil</t>
         </is>
       </c>
     </row>

</xml_diff>